<commit_message>
volver a una sola columna Fecha en la carga por Excel
Rollback de Dia/Mes/Ano a un unico campo Fecha, como era antes. El parser
acepta lo que muestre la celda (dd/mm/aaaa), el ISO tipeado a mano y el
numero de serie de Excel; si viene en mm/dd (Excel en ingles) lo detecta.

La plantilla se regenera con la columna A como celda de fecha real
(DD/MM/AAAA) y el resto de las columnas corridas una posicion.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plantilla-viajes.xlsx
+++ b/public/plantilla-viajes.xlsx
@@ -18,7 +18,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
+  </numFmts>
   <fonts count="5">
     <font>
       <name val="Calibri"/>
@@ -93,12 +96,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -196,20 +205,20 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Dia / Mes / Año: completar solo con numeros (ej: 19 / 6 / 2026).</t>
+        <t>Fecha del viaje en formato DD/MM/AAAA (ej: 19/06/2026).</t>
       </text>
     </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
+    <comment ref="D1" authorId="0" shapeId="0">
       <text>
         <t>Varios pasajeros separados por  |  (ej: M. Rojo | N. Fabbri). Maximo 4.</t>
       </text>
     </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
+    <comment ref="E1" authorId="0" shapeId="0">
       <text>
         <t>Un telefono por pasajero, en el MISMO orden y separados por  |  (ej: +54 9 11 4490-7781 | +54 9 11 6033-2210).</t>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
+    <comment ref="F1" authorId="0" shapeId="0">
       <text>
         <t>Llegada (in) = arribo con vuelo
 Salida (out) = salida con vuelo
@@ -217,7 +226,7 @@
 Otro = traslado</t>
       </text>
     </comment>
-    <comment ref="M1" authorId="0" shapeId="0">
+    <comment ref="K1" authorId="0" shapeId="0">
       <text>
         <t>Destino 2 / Destino 3: tramos adicionales del mismo viaje. Dejar vacio si el viaje tiene un solo tramo.</t>
       </text>
@@ -515,92 +524,80 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
-    <col width="9" customWidth="1" min="11" max="11"/>
-    <col width="26" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
-    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Dia</t>
+          <t>Fecha</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Mes</t>
+          <t>Hora</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Año</t>
+          <t>Categoria</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Hora</t>
+          <t>Pasajeros</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Categoria</t>
+          <t>Telefono</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Pasajeros</t>
+          <t>Tipo</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Telefono</t>
+          <t>Origen</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Tipo</t>
+          <t>Destino</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Origen</t>
+          <t>Vuelo</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Destino</t>
+          <t>Observaciones</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Vuelo</t>
+          <t>Destino 2</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Observaciones</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Destino 2</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Destino 3</t>
         </is>
@@ -608,284 +605,254 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
+        <v>46255</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>07:30</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Ejecutivo</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>JUAN PABLO VOJVODA</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>+54 9 11 5555-1234</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Llegada (in)</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Aeropuerto Ezeiza (EZE)</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>725 Continental</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>AR1234</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="2" t="inlineStr"/>
+      <c r="J2" s="3" t="inlineStr"/>
+      <c r="K2" s="3" t="inlineStr"/>
+      <c r="L2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="B3" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="A3" s="4" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>10:00</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>Auto Std</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>M. ROJO | N. FABBRI</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>+54 9 11 4490-7781 | +54 9 11 6033-2210</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>Salida (out)</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>Santos Dumont 3429</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>Aeropuerto Ezeiza (EZE)</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="I3" s="5" t="inlineStr">
         <is>
           <t>AR1256</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr"/>
-      <c r="M3" s="3" t="inlineStr"/>
-      <c r="N3" s="3" t="inlineStr"/>
+      <c r="J3" s="5" t="inlineStr"/>
+      <c r="K3" s="5" t="inlineStr"/>
+      <c r="L3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
+        <v>46255</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>11:15</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>MB</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>CHAQUEÑO PALAVECINO</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>+54 9 387 555-1456</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Salida (out)</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Balcarce 230, Salta</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Aeropuerto de Salta</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>AR1456</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="inlineStr"/>
-      <c r="N4" s="2" t="inlineStr"/>
+      <c r="J4" s="3" t="inlineStr"/>
+      <c r="K4" s="3" t="inlineStr"/>
+      <c r="L4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="A5" s="4" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>Vito</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>MARTÍN ROMAGNOLI</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>+54 9 11 5555-4302</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>Otro</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>Hotel Faena</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>Hotel Alvear</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr"/>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr"/>
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>Pasa a buscar valijas</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="K5" s="5" t="inlineStr">
         <is>
           <t>San Isidro</t>
         </is>
       </c>
-      <c r="N5" s="3" t="inlineStr"/>
+      <c r="L5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
+        <v>46255</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>10:00</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Ejecutivo</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>F. ACOSTA</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>+54 9 11 5555-7788</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Hs Disposición</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Hotel Alvear</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>Hotel Alvear</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr"/>
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>4 hs a disposicion</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr"/>
-      <c r="N6" s="2" t="inlineStr"/>
+      <c r="K6" s="3" t="inlineStr"/>
+      <c r="L6" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="H2:H200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Elegi un Tipo de la lista." prompt="Elegi: Llegada (in) / Salida (out) / Hs Disposición / Otro" type="list">
+    <dataValidation sqref="F2:F200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Elegi un Tipo de la lista." prompt="Elegi: Llegada (in) / Salida (out) / Hs Disposición / Otro" type="list">
       <formula1>=LOV!$A$2:$A$5</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Elegi una Categoria de la lista." prompt="Elegi: Auto Std / Ejecutivo / MB / Vito" type="list">
+    <dataValidation sqref="C2:C200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Elegi una Categoria de la lista." prompt="Elegi: Auto Std / Ejecutivo / MB / Vito" type="list">
       <formula1>=LOV!$B$2:$B$5</formula1>
     </dataValidation>
   </dataValidations>
@@ -908,12 +875,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Categoria</t>
         </is>
@@ -986,139 +953,139 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Plantilla de carga de viajes</t>
         </is>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Hoja Viajes</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>Una fila por VIAJE. Para tramos adicionales usa las columnas Destino 2 y Destino 3.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>Dia / Mes / Año</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>Completar los tres campos solo con numeros (ej: 19 / 6 / 2026).</t>
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Fecha del viaje en formato DD/MM/AAAA (ej: 19/06/2026).</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Hora</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Formato HH:MM en 24 horas (ej: 07:30).</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Categoria</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>Elegir del desplegable: Auto Std / Ejecutivo / MB / Vito.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Pasajeros</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>Nombre del pasajero. Varios separados con  |  (pipe). Maximo 4.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Telefono</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>OBLIGATORIO. Un telefono por pasajero, en el mismo orden que Pasajeros, separados con  |  (ej: +54 9 11 4490-7781 | +54 9 11 6033-2210).</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Llegada (in) = arribo con vuelo · Salida (out) = salida con vuelo · Hs Disposición = horas a disposicion · Otro = traslado.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>Origen / Destino</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>Direccion o lugar (el sistema usa Google Maps para geolocalizar la direccion).</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>Destino 2 / Destino 3</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>Tramos adicionales del mismo viaje. Dejar vacio si hay un solo tramo.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>Vuelo</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>Solo para tipo Llegada (in) / Salida (out), ej: AR1234. Dejar vacio en otros casos.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>Texto libre opcional.</t>
         </is>

</xml_diff>